<commit_message>
fix: repair leave submission and file upload with fallback, and restore database seed data
</commit_message>
<xml_diff>
--- a/user-credentials.xlsx
+++ b/user-credentials.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="136">
   <si>
     <t>ชื่อ-สกุล</t>
   </si>
@@ -412,6 +412,15 @@
   </si>
   <si>
     <t>69000008@go.buu.ac.th</t>
+  </si>
+  <si>
+    <t>ณภัทร สุขสมบูรณ์</t>
+  </si>
+  <si>
+    <t>67020940</t>
+  </si>
+  <si>
+    <t>67020940@go.buu.ac.th</t>
   </si>
 </sst>
 </file>
@@ -981,7 +990,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1552,6 +1561,23 @@
         <v>5</v>
       </c>
     </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" t="s">
+        <v>134</v>
+      </c>
+      <c r="C34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>